<commit_message>
Add a calculator for calendar and business days in Excel (69cb5328c8ff14ad2d20de06)
</commit_message>
<xml_diff>
--- a/test_output.xlsx
+++ b/test_output.xlsx
@@ -4,14 +4,23 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Timeline" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Date Calculator" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>Starting Date</t>
+  </si>
+  <si>
+    <t>Number of Days</t>
+  </si>
+  <si>
+    <t>Direction</t>
+  </si>
   <si>
     <t>After</t>
   </si>
@@ -20,9 +29,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="mm/dd/yy"/>
-  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -52,10 +58,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -395,27 +400,49 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A10:G11"/>
+  <dimension ref="A3:B8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="10" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C10" s="1">
-        <v>45778</v>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1">
+        <v>46112.2044712037</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
-        <f>IF(ISNUMBER($C$10), WORKDAY($C$10, IF(G15="After", E15, -E15)), "TBD")</f>
-        <v>45792</v>
-      </c>
-      <c r="E11">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4">
         <v>10</v>
       </c>
-      <c r="G11" t="s">
-        <v>0</v>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <f>IF(B5="Before", B3-B4, B3+B4)</f>
+      </c>
+    </row>
+    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <f>IF(B5="Before", WORKDAY(B3, -B4), WORKDAY(B3, B4))</f>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" sqref="B5">
+      <formula1>"Before,After"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Lock disclosure verbiage in Excel and PDF outputs to prevent editing or removal (69cc3116ebbb81046904ea95)
</commit_message>
<xml_diff>
--- a/test_output.xlsx
+++ b/test_output.xlsx
@@ -4,25 +4,28 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Date Calculator" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Sheet 1" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
-    <t>Starting Date</t>
+    <t>Data 1</t>
   </si>
   <si>
-    <t>Number of Days</t>
+    <t>Data 2</t>
   </si>
   <si>
-    <t>Direction</t>
+    <t>Data 3</t>
   </si>
   <si>
-    <t>After</t>
+    <t>Data 4</t>
+  </si>
+  <si>
+    <t>Disclosure</t>
   </si>
 </sst>
 </file>
@@ -58,9 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -400,49 +406,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:B8"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1">
-        <v>46112.2044712037</v>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B7">
-        <f>IF(B5="Before", B3-B4, B3+B4)</f>
-      </c>
-    </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B8">
-        <f>IF(B5="Before", WORKDAY(B3, -B4), WORKDAY(B3, B4))</f>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" sqref="B5">
-      <formula1>"Before,After"</formula1>
-    </dataValidation>
-  </dataValidations>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="L3YXFK1LJhf/rXfDyxDcZ+y2bTcQkYw/Yp5PNcQxXVAyLi8kVixWbfPusqb4jvLCggOcqZkLttXuT0Lm5LBw9A==" saltValue="TgVKbDnEW51ntLVxCmuvIg==" spinCount="100000"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix export issue on fnttimeline.netlify.app to retain Excel formulas (69e7eb2b7d30182ef4fb46f8)
</commit_message>
<xml_diff>
--- a/test_output.xlsx
+++ b/test_output.xlsx
@@ -4,22 +4,16 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Date Calculator" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Timeline" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
-    <t>Starting Date</t>
-  </si>
-  <si>
-    <t>Number of Days</t>
-  </si>
-  <si>
-    <t>Direction</t>
+    <t>Yes</t>
   </si>
   <si>
     <t>After</t>
@@ -29,6 +23,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="mm/dd/yy"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -60,7 +57,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -400,49 +397,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:B8"/>
+  <dimension ref="A10:G12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="10" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C10" s="1">
+        <v>45209</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <f>IF(ISNUMBER($C$10), IF(F12="Yes", WORKDAY($C$10, IF(G12="After", E12, -E12)), IF(G12="After", $C$10 + E12, $C$10 - E12)), "TBD")</f>
+        <v>45223</v>
+      </c>
+      <c r="E12">
+        <v>10</v>
+      </c>
+      <c r="F12" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1">
-        <v>46112.2044712037</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="G12" t="s">
         <v>1</v>
-      </c>
-      <c r="B4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B7">
-        <f>IF(B5="Before", B3-B4, B3+B4)</f>
-      </c>
-    </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B8">
-        <f>IF(B5="Before", WORKDAY(B3, -B4), WORKDAY(B3, B4))</f>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" sqref="B5">
-      <formula1>"Before,After"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>